<commit_message>
feat(modality): drop rationale, add optional Entities suggestions
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/official/create_new_modality/modality_proposal_template.xlsx
+++ b/official/create_new_modality/modality_proposal_template.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modality" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Columns" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Types" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Entities" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -415,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,11 +440,6 @@
           <t>Description</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Rationale</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -464,11 +460,6 @@
       <c r="D2" t="inlineStr">
         <is>
           <t>Venous blood samples drawn alongside MRI</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Blood is drawn at each MRI session; this keeps the analyte values next to the imaging data.</t>
         </is>
       </c>
     </row>
@@ -784,4 +775,69 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Entity</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>acq</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>fasting</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Drawn after at least 8 hours without food</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>acq</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>nonfasting</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Drawn without fasting</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>